<commit_message>
Add new frontend data dictionary file
</commit_message>
<xml_diff>
--- a/R-db2frontend/db2frontend/inst/extdata/Frontend_Table_Description.xlsx
+++ b/R-db2frontend/db2frontend/inst/extdata/Frontend_Table_Description.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="484">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -480,6 +480,36 @@
   </si>
   <si>
     <t xml:space="preserve">5. Medikament ATC / Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_atc1_2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Medikament ATC / Name*:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_atc2_2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Medikament ATC / Name:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_atc3_2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Medikament ATC / Name:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_atc4_2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Medikament ATC / Name:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrp_atc5_2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Medikament ATC / Name:</t>
   </si>
   <si>
     <t xml:space="preserve">mrp_med_prod</t>
@@ -3488,7 +3518,7 @@
         <v>220</v>
       </c>
       <c r="C126" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D126" t="s">
         <v>11</v>
@@ -3499,10 +3529,10 @@
         <v>12</v>
       </c>
       <c r="B127" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C127" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D127" t="s">
         <v>11</v>
@@ -3513,10 +3543,10 @@
         <v>12</v>
       </c>
       <c r="B128" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C128" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D128" t="s">
         <v>11</v>
@@ -3527,10 +3557,10 @@
         <v>12</v>
       </c>
       <c r="B129" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C129" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D129" t="s">
         <v>11</v>
@@ -3541,10 +3571,10 @@
         <v>12</v>
       </c>
       <c r="B130" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C130" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D130" t="s">
         <v>11</v>
@@ -3555,10 +3585,10 @@
         <v>12</v>
       </c>
       <c r="B131" t="s">
+        <v>230</v>
+      </c>
+      <c r="C131" t="s">
         <v>229</v>
-      </c>
-      <c r="C131" t="s">
-        <v>230</v>
       </c>
       <c r="D131" t="s">
         <v>11</v>
@@ -3852,7 +3882,7 @@
         <v>271</v>
       </c>
       <c r="C152" t="s">
-        <v>38</v>
+        <v>272</v>
       </c>
       <c r="D152" t="s">
         <v>11</v>
@@ -3863,10 +3893,10 @@
         <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C153" t="s">
-        <v>40</v>
+        <v>274</v>
       </c>
       <c r="D153" t="s">
         <v>11</v>
@@ -3874,13 +3904,13 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>273</v>
+        <v>12</v>
       </c>
       <c r="B154" t="s">
-        <v>9</v>
+        <v>275</v>
       </c>
       <c r="C154" t="s">
-        <v>10</v>
+        <v>276</v>
       </c>
       <c r="D154" t="s">
         <v>11</v>
@@ -3891,10 +3921,10 @@
         <v>12</v>
       </c>
       <c r="B155" t="s">
-        <v>13</v>
+        <v>277</v>
       </c>
       <c r="C155" t="s">
-        <v>14</v>
+        <v>278</v>
       </c>
       <c r="D155" t="s">
         <v>11</v>
@@ -3905,10 +3935,10 @@
         <v>12</v>
       </c>
       <c r="B156" t="s">
-        <v>15</v>
+        <v>279</v>
       </c>
       <c r="C156" t="s">
-        <v>16</v>
+        <v>280</v>
       </c>
       <c r="D156" t="s">
         <v>11</v>
@@ -3919,10 +3949,10 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>17</v>
+        <v>281</v>
       </c>
       <c r="C157" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D157" t="s">
         <v>11</v>
@@ -3933,10 +3963,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C158" t="s">
-        <v>275</v>
+        <v>40</v>
       </c>
       <c r="D158" t="s">
         <v>11</v>
@@ -3944,13 +3974,13 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>12</v>
+        <v>283</v>
       </c>
       <c r="B159" t="s">
-        <v>276</v>
+        <v>9</v>
       </c>
       <c r="C159" t="s">
-        <v>277</v>
+        <v>10</v>
       </c>
       <c r="D159" t="s">
         <v>11</v>
@@ -3961,10 +3991,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>278</v>
+        <v>13</v>
       </c>
       <c r="C160" t="s">
-        <v>279</v>
+        <v>14</v>
       </c>
       <c r="D160" t="s">
         <v>11</v>
@@ -3975,13 +4005,13 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>280</v>
+        <v>15</v>
       </c>
       <c r="C161" t="s">
-        <v>281</v>
+        <v>16</v>
       </c>
       <c r="D161" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
     </row>
     <row r="162">
@@ -3989,13 +4019,13 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>282</v>
+        <v>17</v>
       </c>
       <c r="C162" t="s">
-        <v>283</v>
+        <v>18</v>
       </c>
       <c r="D162" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
     </row>
     <row r="163">
@@ -4020,7 +4050,7 @@
         <v>286</v>
       </c>
       <c r="C164" t="s">
-        <v>219</v>
+        <v>287</v>
       </c>
       <c r="D164" t="s">
         <v>11</v>
@@ -4031,10 +4061,10 @@
         <v>12</v>
       </c>
       <c r="B165" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C165" t="s">
-        <v>219</v>
+        <v>289</v>
       </c>
       <c r="D165" t="s">
         <v>11</v>
@@ -4045,13 +4075,13 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C166" t="s">
-        <v>147</v>
+        <v>291</v>
       </c>
       <c r="D166" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="167">
@@ -4059,13 +4089,13 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C167" t="s">
-        <v>149</v>
+        <v>293</v>
       </c>
       <c r="D167" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="168">
@@ -4073,10 +4103,10 @@
         <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="C168" t="s">
-        <v>222</v>
+        <v>295</v>
       </c>
       <c r="D168" t="s">
         <v>11</v>
@@ -4087,10 +4117,10 @@
         <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C169" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D169" t="s">
         <v>11</v>
@@ -4101,10 +4131,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C170" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D170" t="s">
         <v>11</v>
@@ -4115,10 +4145,10 @@
         <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C171" t="s">
-        <v>294</v>
+        <v>147</v>
       </c>
       <c r="D171" t="s">
         <v>11</v>
@@ -4129,10 +4159,10 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C172" t="s">
-        <v>296</v>
+        <v>149</v>
       </c>
       <c r="D172" t="s">
         <v>11</v>
@@ -4143,10 +4173,10 @@
         <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C173" t="s">
-        <v>298</v>
+        <v>232</v>
       </c>
       <c r="D173" t="s">
         <v>11</v>
@@ -4157,10 +4187,10 @@
         <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C174" t="s">
-        <v>300</v>
+        <v>234</v>
       </c>
       <c r="D174" t="s">
         <v>11</v>
@@ -4171,10 +4201,10 @@
         <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C175" t="s">
-        <v>302</v>
+        <v>236</v>
       </c>
       <c r="D175" t="s">
         <v>11</v>
@@ -4286,7 +4316,7 @@
         <v>317</v>
       </c>
       <c r="C183" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="D183" t="s">
         <v>11</v>
@@ -4297,10 +4327,10 @@
         <v>12</v>
       </c>
       <c r="B184" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C184" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="D184" t="s">
         <v>11</v>
@@ -4311,10 +4341,10 @@
         <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C185" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="D185" t="s">
         <v>11</v>
@@ -4325,10 +4355,10 @@
         <v>12</v>
       </c>
       <c r="B186" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C186" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="D186" t="s">
         <v>11</v>
@@ -4339,10 +4369,10 @@
         <v>12</v>
       </c>
       <c r="B187" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C187" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="D187" t="s">
         <v>11</v>
@@ -4353,10 +4383,10 @@
         <v>12</v>
       </c>
       <c r="B188" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C188" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D188" t="s">
         <v>11</v>
@@ -4367,10 +4397,10 @@
         <v>12</v>
       </c>
       <c r="B189" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C189" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D189" t="s">
         <v>11</v>
@@ -4381,10 +4411,10 @@
         <v>12</v>
       </c>
       <c r="B190" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C190" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D190" t="s">
         <v>11</v>
@@ -4395,10 +4425,10 @@
         <v>12</v>
       </c>
       <c r="B191" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C191" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D191" t="s">
         <v>11</v>
@@ -4412,7 +4442,7 @@
         <v>331</v>
       </c>
       <c r="C192" t="s">
-        <v>228</v>
+        <v>332</v>
       </c>
       <c r="D192" t="s">
         <v>11</v>
@@ -4423,10 +4453,10 @@
         <v>12</v>
       </c>
       <c r="B193" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C193" t="s">
-        <v>230</v>
+        <v>334</v>
       </c>
       <c r="D193" t="s">
         <v>11</v>
@@ -4437,10 +4467,10 @@
         <v>12</v>
       </c>
       <c r="B194" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C194" t="s">
-        <v>232</v>
+        <v>336</v>
       </c>
       <c r="D194" t="s">
         <v>11</v>
@@ -4451,10 +4481,10 @@
         <v>12</v>
       </c>
       <c r="B195" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C195" t="s">
-        <v>234</v>
+        <v>338</v>
       </c>
       <c r="D195" t="s">
         <v>11</v>
@@ -4465,10 +4495,10 @@
         <v>12</v>
       </c>
       <c r="B196" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C196" t="s">
-        <v>236</v>
+        <v>340</v>
       </c>
       <c r="D196" t="s">
         <v>11</v>
@@ -4479,7 +4509,7 @@
         <v>12</v>
       </c>
       <c r="B197" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C197" t="s">
         <v>238</v>
@@ -4493,7 +4523,7 @@
         <v>12</v>
       </c>
       <c r="B198" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C198" t="s">
         <v>240</v>
@@ -4507,7 +4537,7 @@
         <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="C199" t="s">
         <v>242</v>
@@ -4521,7 +4551,7 @@
         <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C200" t="s">
         <v>244</v>
@@ -4535,7 +4565,7 @@
         <v>12</v>
       </c>
       <c r="B201" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C201" t="s">
         <v>246</v>
@@ -4549,7 +4579,7 @@
         <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="C202" t="s">
         <v>248</v>
@@ -4563,7 +4593,7 @@
         <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C203" t="s">
         <v>250</v>
@@ -4577,7 +4607,7 @@
         <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C204" t="s">
         <v>252</v>
@@ -4591,7 +4621,7 @@
         <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C205" t="s">
         <v>254</v>
@@ -4605,7 +4635,7 @@
         <v>12</v>
       </c>
       <c r="B206" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C206" t="s">
         <v>256</v>
@@ -4619,7 +4649,7 @@
         <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C207" t="s">
         <v>258</v>
@@ -4633,7 +4663,7 @@
         <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="C208" t="s">
         <v>260</v>
@@ -4647,7 +4677,7 @@
         <v>12</v>
       </c>
       <c r="B209" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C209" t="s">
         <v>262</v>
@@ -4661,7 +4691,7 @@
         <v>12</v>
       </c>
       <c r="B210" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="C210" t="s">
         <v>264</v>
@@ -4675,13 +4705,13 @@
         <v>12</v>
       </c>
       <c r="B211" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C211" t="s">
-        <v>351</v>
+        <v>266</v>
       </c>
       <c r="D211" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
     </row>
     <row r="212">
@@ -4689,10 +4719,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C212" t="s">
-        <v>353</v>
+        <v>268</v>
       </c>
       <c r="D212" t="s">
         <v>11</v>
@@ -4703,10 +4733,10 @@
         <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C213" t="s">
-        <v>355</v>
+        <v>270</v>
       </c>
       <c r="D213" t="s">
         <v>11</v>
@@ -4717,10 +4747,10 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C214" t="s">
-        <v>12</v>
+        <v>272</v>
       </c>
       <c r="D214" t="s">
         <v>11</v>
@@ -4731,10 +4761,10 @@
         <v>12</v>
       </c>
       <c r="B215" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C215" t="s">
-        <v>12</v>
+        <v>274</v>
       </c>
       <c r="D215" t="s">
         <v>11</v>
@@ -4745,13 +4775,13 @@
         <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C216" t="s">
-        <v>294</v>
+        <v>361</v>
       </c>
       <c r="D216" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="217">
@@ -4759,10 +4789,10 @@
         <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C217" t="s">
-        <v>296</v>
+        <v>363</v>
       </c>
       <c r="D217" t="s">
         <v>11</v>
@@ -4773,10 +4803,10 @@
         <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C218" t="s">
-        <v>298</v>
+        <v>365</v>
       </c>
       <c r="D218" t="s">
         <v>11</v>
@@ -4787,10 +4817,10 @@
         <v>12</v>
       </c>
       <c r="B219" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="C219" t="s">
-        <v>300</v>
+        <v>12</v>
       </c>
       <c r="D219" t="s">
         <v>11</v>
@@ -4801,10 +4831,10 @@
         <v>12</v>
       </c>
       <c r="B220" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C220" t="s">
-        <v>326</v>
+        <v>12</v>
       </c>
       <c r="D220" t="s">
         <v>11</v>
@@ -4815,10 +4845,10 @@
         <v>12</v>
       </c>
       <c r="B221" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="C221" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D221" t="s">
         <v>11</v>
@@ -4829,10 +4859,10 @@
         <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C222" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D222" t="s">
         <v>11</v>
@@ -4843,10 +4873,10 @@
         <v>12</v>
       </c>
       <c r="B223" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C223" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D223" t="s">
         <v>11</v>
@@ -4857,10 +4887,10 @@
         <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C224" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D224" t="s">
         <v>11</v>
@@ -4871,10 +4901,10 @@
         <v>12</v>
       </c>
       <c r="B225" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="C225" t="s">
-        <v>310</v>
+        <v>336</v>
       </c>
       <c r="D225" t="s">
         <v>11</v>
@@ -4885,7 +4915,7 @@
         <v>12</v>
       </c>
       <c r="B226" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="C226" t="s">
         <v>312</v>
@@ -4899,7 +4929,7 @@
         <v>12</v>
       </c>
       <c r="B227" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="C227" t="s">
         <v>314</v>
@@ -4913,7 +4943,7 @@
         <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="C228" t="s">
         <v>316</v>
@@ -4927,10 +4957,10 @@
         <v>12</v>
       </c>
       <c r="B229" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C229" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="D229" t="s">
         <v>11</v>
@@ -4941,10 +4971,10 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="C230" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="D230" t="s">
         <v>11</v>
@@ -4955,10 +4985,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C231" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="D231" t="s">
         <v>11</v>
@@ -4969,10 +4999,10 @@
         <v>12</v>
       </c>
       <c r="B232" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="C232" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="D232" t="s">
         <v>11</v>
@@ -4983,10 +5013,10 @@
         <v>12</v>
       </c>
       <c r="B233" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="C233" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="D233" t="s">
         <v>11</v>
@@ -4997,10 +5027,10 @@
         <v>12</v>
       </c>
       <c r="B234" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C234" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D234" t="s">
         <v>11</v>
@@ -5011,10 +5041,10 @@
         <v>12</v>
       </c>
       <c r="B235" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C235" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="D235" t="s">
         <v>11</v>
@@ -5025,10 +5055,10 @@
         <v>12</v>
       </c>
       <c r="B236" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C236" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="D236" t="s">
         <v>11</v>
@@ -5039,10 +5069,10 @@
         <v>12</v>
       </c>
       <c r="B237" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="C237" t="s">
-        <v>228</v>
+        <v>326</v>
       </c>
       <c r="D237" t="s">
         <v>11</v>
@@ -5053,10 +5083,10 @@
         <v>12</v>
       </c>
       <c r="B238" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C238" t="s">
-        <v>230</v>
+        <v>332</v>
       </c>
       <c r="D238" t="s">
         <v>11</v>
@@ -5067,10 +5097,10 @@
         <v>12</v>
       </c>
       <c r="B239" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C239" t="s">
-        <v>232</v>
+        <v>334</v>
       </c>
       <c r="D239" t="s">
         <v>11</v>
@@ -5081,10 +5111,10 @@
         <v>12</v>
       </c>
       <c r="B240" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C240" t="s">
-        <v>234</v>
+        <v>338</v>
       </c>
       <c r="D240" t="s">
         <v>11</v>
@@ -5095,10 +5125,10 @@
         <v>12</v>
       </c>
       <c r="B241" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="C241" t="s">
-        <v>236</v>
+        <v>340</v>
       </c>
       <c r="D241" t="s">
         <v>11</v>
@@ -5109,7 +5139,7 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="C242" t="s">
         <v>238</v>
@@ -5123,7 +5153,7 @@
         <v>12</v>
       </c>
       <c r="B243" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C243" t="s">
         <v>240</v>
@@ -5137,7 +5167,7 @@
         <v>12</v>
       </c>
       <c r="B244" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="C244" t="s">
         <v>242</v>
@@ -5151,7 +5181,7 @@
         <v>12</v>
       </c>
       <c r="B245" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="C245" t="s">
         <v>244</v>
@@ -5165,7 +5195,7 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C246" t="s">
         <v>246</v>
@@ -5179,7 +5209,7 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C247" t="s">
         <v>248</v>
@@ -5193,7 +5223,7 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="C248" t="s">
         <v>250</v>
@@ -5207,7 +5237,7 @@
         <v>12</v>
       </c>
       <c r="B249" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C249" t="s">
         <v>252</v>
@@ -5221,7 +5251,7 @@
         <v>12</v>
       </c>
       <c r="B250" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C250" t="s">
         <v>254</v>
@@ -5235,7 +5265,7 @@
         <v>12</v>
       </c>
       <c r="B251" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C251" t="s">
         <v>256</v>
@@ -5249,7 +5279,7 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C252" t="s">
         <v>258</v>
@@ -5263,7 +5293,7 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="C253" t="s">
         <v>260</v>
@@ -5277,7 +5307,7 @@
         <v>12</v>
       </c>
       <c r="B254" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="C254" t="s">
         <v>262</v>
@@ -5291,7 +5321,7 @@
         <v>12</v>
       </c>
       <c r="B255" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C255" t="s">
         <v>264</v>
@@ -5305,10 +5335,10 @@
         <v>12</v>
       </c>
       <c r="B256" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="C256" t="s">
-        <v>38</v>
+        <v>266</v>
       </c>
       <c r="D256" t="s">
         <v>11</v>
@@ -5319,10 +5349,10 @@
         <v>12</v>
       </c>
       <c r="B257" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="C257" t="s">
-        <v>40</v>
+        <v>268</v>
       </c>
       <c r="D257" t="s">
         <v>11</v>
@@ -5330,13 +5360,13 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>400</v>
+        <v>12</v>
       </c>
       <c r="B258" t="s">
-        <v>9</v>
+        <v>405</v>
       </c>
       <c r="C258" t="s">
-        <v>10</v>
+        <v>270</v>
       </c>
       <c r="D258" t="s">
         <v>11</v>
@@ -5347,10 +5377,10 @@
         <v>12</v>
       </c>
       <c r="B259" t="s">
-        <v>13</v>
+        <v>406</v>
       </c>
       <c r="C259" t="s">
-        <v>14</v>
+        <v>272</v>
       </c>
       <c r="D259" t="s">
         <v>11</v>
@@ -5361,10 +5391,10 @@
         <v>12</v>
       </c>
       <c r="B260" t="s">
-        <v>15</v>
+        <v>407</v>
       </c>
       <c r="C260" t="s">
-        <v>16</v>
+        <v>274</v>
       </c>
       <c r="D260" t="s">
         <v>11</v>
@@ -5375,10 +5405,10 @@
         <v>12</v>
       </c>
       <c r="B261" t="s">
-        <v>17</v>
+        <v>408</v>
       </c>
       <c r="C261" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D261" t="s">
         <v>11</v>
@@ -5389,27 +5419,27 @@
         <v>12</v>
       </c>
       <c r="B262" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="C262" t="s">
-        <v>402</v>
+        <v>40</v>
       </c>
       <c r="D262" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>12</v>
+        <v>410</v>
       </c>
       <c r="B263" t="s">
-        <v>403</v>
+        <v>9</v>
       </c>
       <c r="C263" t="s">
-        <v>404</v>
+        <v>10</v>
       </c>
       <c r="D263" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="264">
@@ -5417,13 +5447,13 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>405</v>
+        <v>13</v>
       </c>
       <c r="C264" t="s">
-        <v>406</v>
+        <v>14</v>
       </c>
       <c r="D264" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="265">
@@ -5431,13 +5461,13 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>407</v>
+        <v>15</v>
       </c>
       <c r="C265" t="s">
-        <v>408</v>
+        <v>16</v>
       </c>
       <c r="D265" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="266">
@@ -5445,13 +5475,13 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>409</v>
+        <v>17</v>
       </c>
       <c r="C266" t="s">
-        <v>410</v>
+        <v>18</v>
       </c>
       <c r="D266" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="267">
@@ -5574,24 +5604,24 @@
         <v>427</v>
       </c>
       <c r="C275" t="s">
-        <v>40</v>
+        <v>428</v>
       </c>
       <c r="D275" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>428</v>
+        <v>12</v>
       </c>
       <c r="B276" t="s">
-        <v>9</v>
+        <v>429</v>
       </c>
       <c r="C276" t="s">
-        <v>10</v>
+        <v>430</v>
       </c>
       <c r="D276" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="277">
@@ -5599,13 +5629,13 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>13</v>
+        <v>431</v>
       </c>
       <c r="C277" t="s">
-        <v>14</v>
+        <v>432</v>
       </c>
       <c r="D277" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="278">
@@ -5613,13 +5643,13 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>15</v>
+        <v>433</v>
       </c>
       <c r="C278" t="s">
-        <v>16</v>
+        <v>434</v>
       </c>
       <c r="D278" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="279">
@@ -5627,13 +5657,13 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>17</v>
+        <v>435</v>
       </c>
       <c r="C279" t="s">
-        <v>18</v>
+        <v>436</v>
       </c>
       <c r="D279" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="280">
@@ -5641,27 +5671,27 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C280" t="s">
-        <v>430</v>
+        <v>40</v>
       </c>
       <c r="D280" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>12</v>
+        <v>438</v>
       </c>
       <c r="B281" t="s">
-        <v>431</v>
+        <v>9</v>
       </c>
       <c r="C281" t="s">
-        <v>432</v>
+        <v>10</v>
       </c>
       <c r="D281" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="282">
@@ -5669,13 +5699,13 @@
         <v>12</v>
       </c>
       <c r="B282" t="s">
-        <v>433</v>
+        <v>13</v>
       </c>
       <c r="C282" t="s">
-        <v>434</v>
+        <v>14</v>
       </c>
       <c r="D282" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="283">
@@ -5683,13 +5713,13 @@
         <v>12</v>
       </c>
       <c r="B283" t="s">
-        <v>435</v>
+        <v>15</v>
       </c>
       <c r="C283" t="s">
-        <v>436</v>
+        <v>16</v>
       </c>
       <c r="D283" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="284">
@@ -5697,13 +5727,13 @@
         <v>12</v>
       </c>
       <c r="B284" t="s">
-        <v>437</v>
+        <v>17</v>
       </c>
       <c r="C284" t="s">
-        <v>438</v>
+        <v>18</v>
       </c>
       <c r="D284" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="285">
@@ -5952,9 +5982,79 @@
         <v>473</v>
       </c>
       <c r="C302" t="s">
+        <v>474</v>
+      </c>
+      <c r="D302" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="s">
+        <v>12</v>
+      </c>
+      <c r="B303" t="s">
+        <v>475</v>
+      </c>
+      <c r="C303" t="s">
+        <v>476</v>
+      </c>
+      <c r="D303" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="s">
+        <v>12</v>
+      </c>
+      <c r="B304" t="s">
+        <v>477</v>
+      </c>
+      <c r="C304" t="s">
+        <v>478</v>
+      </c>
+      <c r="D304" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="s">
+        <v>12</v>
+      </c>
+      <c r="B305" t="s">
+        <v>479</v>
+      </c>
+      <c r="C305" t="s">
+        <v>480</v>
+      </c>
+      <c r="D305" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="s">
+        <v>12</v>
+      </c>
+      <c r="B306" t="s">
+        <v>481</v>
+      </c>
+      <c r="C306" t="s">
+        <v>482</v>
+      </c>
+      <c r="D306" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="s">
+        <v>12</v>
+      </c>
+      <c r="B307" t="s">
+        <v>483</v>
+      </c>
+      <c r="C307" t="s">
         <v>40</v>
       </c>
-      <c r="D302" t="s">
+      <c r="D307" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Frontend_Table_Description and SQL files
</commit_message>
<xml_diff>
--- a/R-db2frontend/db2frontend/inst/extdata/Frontend_Table_Description.xlsx
+++ b/R-db2frontend/db2frontend/inst/extdata/Frontend_Table_Description.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="489">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -947,6 +947,9 @@
     <t xml:space="preserve">Grund für nicht Bestätigung</t>
   </si>
   <si>
+    <t xml:space="preserve">ret_gewiss_grund1_abl_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">ret_gewiss_trigger1_falsch___1</t>
   </si>
   <si>
@@ -1019,6 +1022,12 @@
     <t xml:space="preserve">Kommentar (2. Trigger)</t>
   </si>
   <si>
+    <t xml:space="preserve">ret_gewiss_mrpkonzept1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WELCHE Indikatoren sind zu unspezifisch für den MRP-Trigger und warum?</t>
+  </si>
+  <si>
     <t xml:space="preserve">ret_gewiss_grund_abl_sonst1</t>
   </si>
   <si>
@@ -1130,6 +1139,9 @@
     <t xml:space="preserve">ret_gewiss_grund2_abl</t>
   </si>
   <si>
+    <t xml:space="preserve">ret_gewiss_grund2_abl_01</t>
+  </si>
+  <si>
     <t xml:space="preserve">ret_gewiss_grund_abl_sonst2</t>
   </si>
   <si>
@@ -1173,6 +1185,9 @@
   </si>
   <si>
     <t xml:space="preserve">ret_gewiss_datengrundl2_2_oth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ret_gewiss_mrpkonzept2</t>
   </si>
   <si>
     <t xml:space="preserve">ret_gewiss_grund_abl_klin2</t>
@@ -4274,7 +4289,7 @@
         <v>311</v>
       </c>
       <c r="C180" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D180" t="s">
         <v>11</v>
@@ -4285,10 +4300,10 @@
         <v>12</v>
       </c>
       <c r="B181" t="s">
+        <v>312</v>
+      </c>
+      <c r="C181" t="s">
         <v>313</v>
-      </c>
-      <c r="C181" t="s">
-        <v>314</v>
       </c>
       <c r="D181" t="s">
         <v>11</v>
@@ -4299,10 +4314,10 @@
         <v>12</v>
       </c>
       <c r="B182" t="s">
+        <v>314</v>
+      </c>
+      <c r="C182" t="s">
         <v>315</v>
-      </c>
-      <c r="C182" t="s">
-        <v>316</v>
       </c>
       <c r="D182" t="s">
         <v>11</v>
@@ -4313,10 +4328,10 @@
         <v>12</v>
       </c>
       <c r="B183" t="s">
+        <v>316</v>
+      </c>
+      <c r="C183" t="s">
         <v>317</v>
-      </c>
-      <c r="C183" t="s">
-        <v>318</v>
       </c>
       <c r="D183" t="s">
         <v>11</v>
@@ -4327,10 +4342,10 @@
         <v>12</v>
       </c>
       <c r="B184" t="s">
+        <v>318</v>
+      </c>
+      <c r="C184" t="s">
         <v>319</v>
-      </c>
-      <c r="C184" t="s">
-        <v>320</v>
       </c>
       <c r="D184" t="s">
         <v>11</v>
@@ -4341,10 +4356,10 @@
         <v>12</v>
       </c>
       <c r="B185" t="s">
+        <v>320</v>
+      </c>
+      <c r="C185" t="s">
         <v>321</v>
-      </c>
-      <c r="C185" t="s">
-        <v>322</v>
       </c>
       <c r="D185" t="s">
         <v>11</v>
@@ -4355,10 +4370,10 @@
         <v>12</v>
       </c>
       <c r="B186" t="s">
+        <v>322</v>
+      </c>
+      <c r="C186" t="s">
         <v>323</v>
-      </c>
-      <c r="C186" t="s">
-        <v>324</v>
       </c>
       <c r="D186" t="s">
         <v>11</v>
@@ -4369,10 +4384,10 @@
         <v>12</v>
       </c>
       <c r="B187" t="s">
+        <v>324</v>
+      </c>
+      <c r="C187" t="s">
         <v>325</v>
-      </c>
-      <c r="C187" t="s">
-        <v>326</v>
       </c>
       <c r="D187" t="s">
         <v>11</v>
@@ -4383,10 +4398,10 @@
         <v>12</v>
       </c>
       <c r="B188" t="s">
+        <v>326</v>
+      </c>
+      <c r="C188" t="s">
         <v>327</v>
-      </c>
-      <c r="C188" t="s">
-        <v>320</v>
       </c>
       <c r="D188" t="s">
         <v>11</v>
@@ -4400,7 +4415,7 @@
         <v>328</v>
       </c>
       <c r="C189" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D189" t="s">
         <v>11</v>
@@ -4414,7 +4429,7 @@
         <v>329</v>
       </c>
       <c r="C190" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D190" t="s">
         <v>11</v>
@@ -4428,7 +4443,7 @@
         <v>330</v>
       </c>
       <c r="C191" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D191" t="s">
         <v>11</v>
@@ -4442,7 +4457,7 @@
         <v>331</v>
       </c>
       <c r="C192" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="D192" t="s">
         <v>11</v>
@@ -4453,10 +4468,10 @@
         <v>12</v>
       </c>
       <c r="B193" t="s">
+        <v>332</v>
+      </c>
+      <c r="C193" t="s">
         <v>333</v>
-      </c>
-      <c r="C193" t="s">
-        <v>334</v>
       </c>
       <c r="D193" t="s">
         <v>11</v>
@@ -4467,10 +4482,10 @@
         <v>12</v>
       </c>
       <c r="B194" t="s">
+        <v>334</v>
+      </c>
+      <c r="C194" t="s">
         <v>335</v>
-      </c>
-      <c r="C194" t="s">
-        <v>336</v>
       </c>
       <c r="D194" t="s">
         <v>11</v>
@@ -4481,10 +4496,10 @@
         <v>12</v>
       </c>
       <c r="B195" t="s">
+        <v>336</v>
+      </c>
+      <c r="C195" t="s">
         <v>337</v>
-      </c>
-      <c r="C195" t="s">
-        <v>338</v>
       </c>
       <c r="D195" t="s">
         <v>11</v>
@@ -4495,10 +4510,10 @@
         <v>12</v>
       </c>
       <c r="B196" t="s">
+        <v>338</v>
+      </c>
+      <c r="C196" t="s">
         <v>339</v>
-      </c>
-      <c r="C196" t="s">
-        <v>340</v>
       </c>
       <c r="D196" t="s">
         <v>11</v>
@@ -4509,10 +4524,10 @@
         <v>12</v>
       </c>
       <c r="B197" t="s">
+        <v>340</v>
+      </c>
+      <c r="C197" t="s">
         <v>341</v>
-      </c>
-      <c r="C197" t="s">
-        <v>238</v>
       </c>
       <c r="D197" t="s">
         <v>11</v>
@@ -4526,7 +4541,7 @@
         <v>342</v>
       </c>
       <c r="C198" t="s">
-        <v>240</v>
+        <v>343</v>
       </c>
       <c r="D198" t="s">
         <v>11</v>
@@ -4537,10 +4552,10 @@
         <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C199" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D199" t="s">
         <v>11</v>
@@ -4551,10 +4566,10 @@
         <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C200" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D200" t="s">
         <v>11</v>
@@ -4565,10 +4580,10 @@
         <v>12</v>
       </c>
       <c r="B201" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C201" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D201" t="s">
         <v>11</v>
@@ -4579,10 +4594,10 @@
         <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C202" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D202" t="s">
         <v>11</v>
@@ -4593,10 +4608,10 @@
         <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C203" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D203" t="s">
         <v>11</v>
@@ -4607,10 +4622,10 @@
         <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C204" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D204" t="s">
         <v>11</v>
@@ -4621,10 +4636,10 @@
         <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C205" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="D205" t="s">
         <v>11</v>
@@ -4635,10 +4650,10 @@
         <v>12</v>
       </c>
       <c r="B206" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C206" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="D206" t="s">
         <v>11</v>
@@ -4649,10 +4664,10 @@
         <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C207" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D207" t="s">
         <v>11</v>
@@ -4663,10 +4678,10 @@
         <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C208" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D208" t="s">
         <v>11</v>
@@ -4677,10 +4692,10 @@
         <v>12</v>
       </c>
       <c r="B209" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C209" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D209" t="s">
         <v>11</v>
@@ -4691,10 +4706,10 @@
         <v>12</v>
       </c>
       <c r="B210" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C210" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="D210" t="s">
         <v>11</v>
@@ -4705,10 +4720,10 @@
         <v>12</v>
       </c>
       <c r="B211" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C211" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D211" t="s">
         <v>11</v>
@@ -4719,10 +4734,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C212" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D212" t="s">
         <v>11</v>
@@ -4733,10 +4748,10 @@
         <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C213" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D213" t="s">
         <v>11</v>
@@ -4747,10 +4762,10 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C214" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="D214" t="s">
         <v>11</v>
@@ -4761,10 +4776,10 @@
         <v>12</v>
       </c>
       <c r="B215" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C215" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D215" t="s">
         <v>11</v>
@@ -4775,13 +4790,13 @@
         <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C216" t="s">
-        <v>361</v>
+        <v>272</v>
       </c>
       <c r="D216" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
     </row>
     <row r="217">
@@ -4792,7 +4807,7 @@
         <v>362</v>
       </c>
       <c r="C217" t="s">
-        <v>363</v>
+        <v>274</v>
       </c>
       <c r="D217" t="s">
         <v>11</v>
@@ -4803,13 +4818,13 @@
         <v>12</v>
       </c>
       <c r="B218" t="s">
+        <v>363</v>
+      </c>
+      <c r="C218" t="s">
         <v>364</v>
       </c>
-      <c r="C218" t="s">
-        <v>365</v>
-      </c>
       <c r="D218" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="219">
@@ -4817,10 +4832,10 @@
         <v>12</v>
       </c>
       <c r="B219" t="s">
+        <v>365</v>
+      </c>
+      <c r="C219" t="s">
         <v>366</v>
-      </c>
-      <c r="C219" t="s">
-        <v>12</v>
       </c>
       <c r="D219" t="s">
         <v>11</v>
@@ -4834,7 +4849,7 @@
         <v>367</v>
       </c>
       <c r="C220" t="s">
-        <v>12</v>
+        <v>368</v>
       </c>
       <c r="D220" t="s">
         <v>11</v>
@@ -4845,10 +4860,10 @@
         <v>12</v>
       </c>
       <c r="B221" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C221" t="s">
-        <v>304</v>
+        <v>12</v>
       </c>
       <c r="D221" t="s">
         <v>11</v>
@@ -4859,10 +4874,10 @@
         <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C222" t="s">
-        <v>306</v>
+        <v>12</v>
       </c>
       <c r="D222" t="s">
         <v>11</v>
@@ -4873,10 +4888,10 @@
         <v>12</v>
       </c>
       <c r="B223" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C223" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D223" t="s">
         <v>11</v>
@@ -4887,10 +4902,10 @@
         <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C224" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="D224" t="s">
         <v>11</v>
@@ -4901,10 +4916,10 @@
         <v>12</v>
       </c>
       <c r="B225" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C225" t="s">
-        <v>336</v>
+        <v>308</v>
       </c>
       <c r="D225" t="s">
         <v>11</v>
@@ -4915,10 +4930,10 @@
         <v>12</v>
       </c>
       <c r="B226" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C226" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D226" t="s">
         <v>11</v>
@@ -4929,10 +4944,10 @@
         <v>12</v>
       </c>
       <c r="B227" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C227" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="D227" t="s">
         <v>11</v>
@@ -4943,10 +4958,10 @@
         <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C228" t="s">
-        <v>316</v>
+        <v>339</v>
       </c>
       <c r="D228" t="s">
         <v>11</v>
@@ -4957,10 +4972,10 @@
         <v>12</v>
       </c>
       <c r="B229" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C229" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="D229" t="s">
         <v>11</v>
@@ -4971,10 +4986,10 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C230" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D230" t="s">
         <v>11</v>
@@ -4985,10 +5000,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C231" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D231" t="s">
         <v>11</v>
@@ -4999,10 +5014,10 @@
         <v>12</v>
       </c>
       <c r="B232" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C232" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D232" t="s">
         <v>11</v>
@@ -5013,10 +5028,10 @@
         <v>12</v>
       </c>
       <c r="B233" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C233" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D233" t="s">
         <v>11</v>
@@ -5027,10 +5042,10 @@
         <v>12</v>
       </c>
       <c r="B234" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C234" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="D234" t="s">
         <v>11</v>
@@ -5041,10 +5056,10 @@
         <v>12</v>
       </c>
       <c r="B235" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C235" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D235" t="s">
         <v>11</v>
@@ -5055,10 +5070,10 @@
         <v>12</v>
       </c>
       <c r="B236" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C236" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D236" t="s">
         <v>11</v>
@@ -5069,10 +5084,10 @@
         <v>12</v>
       </c>
       <c r="B237" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C237" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D237" t="s">
         <v>11</v>
@@ -5083,10 +5098,10 @@
         <v>12</v>
       </c>
       <c r="B238" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C238" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="D238" t="s">
         <v>11</v>
@@ -5097,10 +5112,10 @@
         <v>12</v>
       </c>
       <c r="B239" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C239" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="D239" t="s">
         <v>11</v>
@@ -5111,10 +5126,10 @@
         <v>12</v>
       </c>
       <c r="B240" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C240" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="D240" t="s">
         <v>11</v>
@@ -5125,10 +5140,10 @@
         <v>12</v>
       </c>
       <c r="B241" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C241" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="D241" t="s">
         <v>11</v>
@@ -5139,10 +5154,10 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C242" t="s">
-        <v>238</v>
+        <v>335</v>
       </c>
       <c r="D242" t="s">
         <v>11</v>
@@ -5153,10 +5168,10 @@
         <v>12</v>
       </c>
       <c r="B243" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C243" t="s">
-        <v>240</v>
+        <v>337</v>
       </c>
       <c r="D243" t="s">
         <v>11</v>
@@ -5167,10 +5182,10 @@
         <v>12</v>
       </c>
       <c r="B244" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C244" t="s">
-        <v>242</v>
+        <v>341</v>
       </c>
       <c r="D244" t="s">
         <v>11</v>
@@ -5181,10 +5196,10 @@
         <v>12</v>
       </c>
       <c r="B245" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C245" t="s">
-        <v>244</v>
+        <v>343</v>
       </c>
       <c r="D245" t="s">
         <v>11</v>
@@ -5195,10 +5210,10 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C246" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="D246" t="s">
         <v>11</v>
@@ -5209,10 +5224,10 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C247" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="D247" t="s">
         <v>11</v>
@@ -5223,10 +5238,10 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C248" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="D248" t="s">
         <v>11</v>
@@ -5237,10 +5252,10 @@
         <v>12</v>
       </c>
       <c r="B249" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C249" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="D249" t="s">
         <v>11</v>
@@ -5251,10 +5266,10 @@
         <v>12</v>
       </c>
       <c r="B250" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C250" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="D250" t="s">
         <v>11</v>
@@ -5265,10 +5280,10 @@
         <v>12</v>
       </c>
       <c r="B251" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C251" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="D251" t="s">
         <v>11</v>
@@ -5279,10 +5294,10 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C252" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D252" t="s">
         <v>11</v>
@@ -5293,10 +5308,10 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C253" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="D253" t="s">
         <v>11</v>
@@ -5307,10 +5322,10 @@
         <v>12</v>
       </c>
       <c r="B254" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C254" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="D254" t="s">
         <v>11</v>
@@ -5321,10 +5336,10 @@
         <v>12</v>
       </c>
       <c r="B255" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C255" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D255" t="s">
         <v>11</v>
@@ -5335,10 +5350,10 @@
         <v>12</v>
       </c>
       <c r="B256" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C256" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="D256" t="s">
         <v>11</v>
@@ -5349,10 +5364,10 @@
         <v>12</v>
       </c>
       <c r="B257" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C257" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="D257" t="s">
         <v>11</v>
@@ -5363,10 +5378,10 @@
         <v>12</v>
       </c>
       <c r="B258" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C258" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="D258" t="s">
         <v>11</v>
@@ -5377,10 +5392,10 @@
         <v>12</v>
       </c>
       <c r="B259" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C259" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="D259" t="s">
         <v>11</v>
@@ -5391,10 +5406,10 @@
         <v>12</v>
       </c>
       <c r="B260" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C260" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="D260" t="s">
         <v>11</v>
@@ -5405,10 +5420,10 @@
         <v>12</v>
       </c>
       <c r="B261" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C261" t="s">
-        <v>38</v>
+        <v>268</v>
       </c>
       <c r="D261" t="s">
         <v>11</v>
@@ -5419,10 +5434,10 @@
         <v>12</v>
       </c>
       <c r="B262" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C262" t="s">
-        <v>40</v>
+        <v>270</v>
       </c>
       <c r="D262" t="s">
         <v>11</v>
@@ -5430,13 +5445,13 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>410</v>
+        <v>12</v>
       </c>
       <c r="B263" t="s">
-        <v>9</v>
+        <v>411</v>
       </c>
       <c r="C263" t="s">
-        <v>10</v>
+        <v>272</v>
       </c>
       <c r="D263" t="s">
         <v>11</v>
@@ -5447,10 +5462,10 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>13</v>
+        <v>412</v>
       </c>
       <c r="C264" t="s">
-        <v>14</v>
+        <v>274</v>
       </c>
       <c r="D264" t="s">
         <v>11</v>
@@ -5461,10 +5476,10 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>15</v>
+        <v>413</v>
       </c>
       <c r="C265" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D265" t="s">
         <v>11</v>
@@ -5475,10 +5490,10 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>17</v>
+        <v>414</v>
       </c>
       <c r="C266" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D266" t="s">
         <v>11</v>
@@ -5486,16 +5501,16 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>12</v>
+        <v>415</v>
       </c>
       <c r="B267" t="s">
-        <v>411</v>
+        <v>9</v>
       </c>
       <c r="C267" t="s">
-        <v>412</v>
+        <v>10</v>
       </c>
       <c r="D267" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="268">
@@ -5503,13 +5518,13 @@
         <v>12</v>
       </c>
       <c r="B268" t="s">
-        <v>413</v>
+        <v>13</v>
       </c>
       <c r="C268" t="s">
-        <v>414</v>
+        <v>14</v>
       </c>
       <c r="D268" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="269">
@@ -5517,13 +5532,13 @@
         <v>12</v>
       </c>
       <c r="B269" t="s">
-        <v>415</v>
+        <v>15</v>
       </c>
       <c r="C269" t="s">
-        <v>416</v>
+        <v>16</v>
       </c>
       <c r="D269" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="270">
@@ -5531,13 +5546,13 @@
         <v>12</v>
       </c>
       <c r="B270" t="s">
-        <v>417</v>
+        <v>17</v>
       </c>
       <c r="C270" t="s">
-        <v>418</v>
+        <v>18</v>
       </c>
       <c r="D270" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="271">
@@ -5545,10 +5560,10 @@
         <v>12</v>
       </c>
       <c r="B271" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C271" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D271" t="s">
         <v>48</v>
@@ -5559,10 +5574,10 @@
         <v>12</v>
       </c>
       <c r="B272" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C272" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D272" t="s">
         <v>48</v>
@@ -5573,10 +5588,10 @@
         <v>12</v>
       </c>
       <c r="B273" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C273" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="D273" t="s">
         <v>48</v>
@@ -5587,10 +5602,10 @@
         <v>12</v>
       </c>
       <c r="B274" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C274" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D274" t="s">
         <v>48</v>
@@ -5601,10 +5616,10 @@
         <v>12</v>
       </c>
       <c r="B275" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C275" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="D275" t="s">
         <v>48</v>
@@ -5615,10 +5630,10 @@
         <v>12</v>
       </c>
       <c r="B276" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C276" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="D276" t="s">
         <v>48</v>
@@ -5629,10 +5644,10 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C277" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="D277" t="s">
         <v>48</v>
@@ -5643,10 +5658,10 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C278" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D278" t="s">
         <v>48</v>
@@ -5657,10 +5672,10 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C279" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D279" t="s">
         <v>48</v>
@@ -5671,27 +5686,27 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C280" t="s">
-        <v>40</v>
+        <v>435</v>
       </c>
       <c r="D280" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>438</v>
+        <v>12</v>
       </c>
       <c r="B281" t="s">
-        <v>9</v>
+        <v>436</v>
       </c>
       <c r="C281" t="s">
-        <v>10</v>
+        <v>437</v>
       </c>
       <c r="D281" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="282">
@@ -5699,13 +5714,13 @@
         <v>12</v>
       </c>
       <c r="B282" t="s">
-        <v>13</v>
+        <v>438</v>
       </c>
       <c r="C282" t="s">
-        <v>14</v>
+        <v>439</v>
       </c>
       <c r="D282" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="283">
@@ -5713,13 +5728,13 @@
         <v>12</v>
       </c>
       <c r="B283" t="s">
-        <v>15</v>
+        <v>440</v>
       </c>
       <c r="C283" t="s">
-        <v>16</v>
+        <v>441</v>
       </c>
       <c r="D283" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="284">
@@ -5727,10 +5742,10 @@
         <v>12</v>
       </c>
       <c r="B284" t="s">
-        <v>17</v>
+        <v>442</v>
       </c>
       <c r="C284" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D284" t="s">
         <v>11</v>
@@ -5738,16 +5753,16 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>12</v>
+        <v>443</v>
       </c>
       <c r="B285" t="s">
-        <v>439</v>
+        <v>9</v>
       </c>
       <c r="C285" t="s">
-        <v>440</v>
+        <v>10</v>
       </c>
       <c r="D285" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="286">
@@ -5755,13 +5770,13 @@
         <v>12</v>
       </c>
       <c r="B286" t="s">
-        <v>441</v>
+        <v>13</v>
       </c>
       <c r="C286" t="s">
-        <v>442</v>
+        <v>14</v>
       </c>
       <c r="D286" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="287">
@@ -5769,13 +5784,13 @@
         <v>12</v>
       </c>
       <c r="B287" t="s">
-        <v>443</v>
+        <v>15</v>
       </c>
       <c r="C287" t="s">
-        <v>444</v>
+        <v>16</v>
       </c>
       <c r="D287" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="288">
@@ -5783,13 +5798,13 @@
         <v>12</v>
       </c>
       <c r="B288" t="s">
-        <v>445</v>
+        <v>17</v>
       </c>
       <c r="C288" t="s">
-        <v>446</v>
+        <v>18</v>
       </c>
       <c r="D288" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="289">
@@ -5797,10 +5812,10 @@
         <v>12</v>
       </c>
       <c r="B289" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C289" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="D289" t="s">
         <v>48</v>
@@ -5811,10 +5826,10 @@
         <v>12</v>
       </c>
       <c r="B290" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="C290" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="D290" t="s">
         <v>48</v>
@@ -5825,10 +5840,10 @@
         <v>12</v>
       </c>
       <c r="B291" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="C291" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D291" t="s">
         <v>48</v>
@@ -5839,10 +5854,10 @@
         <v>12</v>
       </c>
       <c r="B292" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="C292" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D292" t="s">
         <v>48</v>
@@ -5853,10 +5868,10 @@
         <v>12</v>
       </c>
       <c r="B293" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C293" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D293" t="s">
         <v>48</v>
@@ -5867,10 +5882,10 @@
         <v>12</v>
       </c>
       <c r="B294" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C294" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="D294" t="s">
         <v>48</v>
@@ -5881,10 +5896,10 @@
         <v>12</v>
       </c>
       <c r="B295" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="C295" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D295" t="s">
         <v>48</v>
@@ -5895,10 +5910,10 @@
         <v>12</v>
       </c>
       <c r="B296" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C296" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="D296" t="s">
         <v>48</v>
@@ -5909,10 +5924,10 @@
         <v>12</v>
       </c>
       <c r="B297" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="C297" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D297" t="s">
         <v>48</v>
@@ -5923,10 +5938,10 @@
         <v>12</v>
       </c>
       <c r="B298" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C298" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D298" t="s">
         <v>48</v>
@@ -5937,10 +5952,10 @@
         <v>12</v>
       </c>
       <c r="B299" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="C299" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D299" t="s">
         <v>48</v>
@@ -5951,10 +5966,10 @@
         <v>12</v>
       </c>
       <c r="B300" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C300" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D300" t="s">
         <v>48</v>
@@ -5965,10 +5980,10 @@
         <v>12</v>
       </c>
       <c r="B301" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="C301" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="D301" t="s">
         <v>48</v>
@@ -5979,10 +5994,10 @@
         <v>12</v>
       </c>
       <c r="B302" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="C302" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="D302" t="s">
         <v>48</v>
@@ -5993,10 +6008,10 @@
         <v>12</v>
       </c>
       <c r="B303" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="C303" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="D303" t="s">
         <v>48</v>
@@ -6007,10 +6022,10 @@
         <v>12</v>
       </c>
       <c r="B304" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="C304" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="D304" t="s">
         <v>48</v>
@@ -6021,10 +6036,10 @@
         <v>12</v>
       </c>
       <c r="B305" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="C305" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="D305" t="s">
         <v>48</v>
@@ -6035,10 +6050,10 @@
         <v>12</v>
       </c>
       <c r="B306" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="C306" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D306" t="s">
         <v>48</v>
@@ -6049,12 +6064,68 @@
         <v>12</v>
       </c>
       <c r="B307" t="s">
+        <v>480</v>
+      </c>
+      <c r="C307" t="s">
+        <v>481</v>
+      </c>
+      <c r="D307" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="s">
+        <v>12</v>
+      </c>
+      <c r="B308" t="s">
+        <v>482</v>
+      </c>
+      <c r="C308" t="s">
         <v>483</v>
       </c>
-      <c r="C307" t="s">
+      <c r="D308" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="s">
+        <v>12</v>
+      </c>
+      <c r="B309" t="s">
+        <v>484</v>
+      </c>
+      <c r="C309" t="s">
+        <v>485</v>
+      </c>
+      <c r="D309" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="s">
+        <v>12</v>
+      </c>
+      <c r="B310" t="s">
+        <v>486</v>
+      </c>
+      <c r="C310" t="s">
+        <v>487</v>
+      </c>
+      <c r="D310" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="s">
+        <v>12</v>
+      </c>
+      <c r="B311" t="s">
+        <v>488</v>
+      </c>
+      <c r="C311" t="s">
         <v>40</v>
       </c>
-      <c r="D307" t="s">
+      <c r="D311" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>